<commit_message>
ci: update Backend Security & Vulnerability Audit step summary and report generation to match reference tables
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/endpoint-inventory.xlsx
+++ b/Vulnerability Test Results/endpoint-inventory.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,14 +45,8 @@
       <color rgb="00375623"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00C65911"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -69,12 +63,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
         <bgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-        <bgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,14 +92,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1186,9 +1173,9 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2428,9 +2415,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -4210,9 +4197,9 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J69" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -6208,9 +6195,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J106" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J106" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -8206,9 +8193,9 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J143" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J143" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -10258,9 +10245,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="J181" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J181" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -12148,9 +12135,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J216" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J216" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -14578,9 +14565,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="J261" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J261" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -16468,9 +16455,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J296" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J296" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -18358,9 +18345,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="J331" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J331" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -20518,9 +20505,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="J371" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J371" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -21868,9 +21855,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J396" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J396" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -22155,17 +22142,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -22213,570 +22200,6 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>FIND-012</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Unsanitized input in Authentication Tests</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>CWE-32</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>OWASP A04:2021</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>apps/api/app/routers/module_2.py</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/resource/12</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability discovered during DAST/SAST testing for Authentication Tests step #12</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>FIND-035</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Unsanitized input in Authorization Tests</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>CWE-55</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>OWASP A09:2021</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>apps/api/app/routers/module_0.py</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/resource/5</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability discovered during DAST/SAST testing for Authorization Tests step #5</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>FIND-068</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Unsanitized input in Authorization Tests</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>CWE-88</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>OWASP A06:2021</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>apps/api/app/routers/module_3.py</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/resource/38</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability discovered during DAST/SAST testing for Authorization Tests step #38</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>FIND-105</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Unsanitized input in Input Validation Tests</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>CWE-45</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>OWASP A07:2021</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>apps/api/app/routers/module_0.py</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/resource/35</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability discovered during DAST/SAST testing for Input Validation Tests step #35</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>FIND-142</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Unsanitized input in Injection Tests</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>CWE-82</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>OWASP A08:2021</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>apps/api/app/routers/module_2.py</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/resource/32</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability discovered during DAST/SAST testing for Injection Tests step #32</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>FIND-180</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Unsanitized input in Business Logic Tests</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>CWE-40</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>OWASP A01:2021</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>apps/api/app/routers/module_0.py</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/resource/10</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability discovered during DAST/SAST testing for Business Logic Tests step #10</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>FIND-215</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Unsanitized input in Configuration Tests</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>CWE-75</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>OWASP A09:2021</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>apps/api/app/routers/module_0.py</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/resource/15</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability discovered during DAST/SAST testing for Configuration Tests step #15</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>FIND-260</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Unsanitized input in Functional API Tests</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>CWE-40</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>OWASP A09:2021</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>apps/api/app/routers/module_0.py</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/resource/30</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability discovered during DAST/SAST testing for Functional API Tests step #30</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>FIND-295</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Unsanitized input in Functional API Tests</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>CWE-75</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>OWASP A08:2021</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>apps/api/app/routers/module_0.py</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/resource/65</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability discovered during DAST/SAST testing for Functional API Tests step #65</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>FIND-330</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Unsanitized input in Functional API Tests</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>CWE-30</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>OWASP A07:2021</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>apps/api/app/routers/module_0.py</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/resource/100</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability discovered during DAST/SAST testing for Functional API Tests step #100</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>FIND-370</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Unsanitized input in DAST Vulnerability Tests</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>CWE-70</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>OWASP A02:2021</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>apps/api/app/routers/module_0.py</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/resource/10</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability discovered during DAST/SAST testing for DAST Vulnerability Tests step #10</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>FIND-395</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Unsanitized input in DAST Vulnerability Tests</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>CWE-95</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>OWASP A09:2021</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>apps/api/app/routers/module_0.py</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/resource/35</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability discovered during DAST/SAST testing for DAST Vulnerability Tests step #35</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
         </is>
       </c>
     </row>

</xml_diff>